<commit_message>
S32: add INLAY (RESIN) 26/10 (84 labor hours)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HsFNnGJRzg6EEfnut1VvMX
</commit_message>
<xml_diff>
--- a/loss-time/outputs/Loss_time_S32_05-10_den_29-10.xlsx
+++ b/loss-time/outputs/Loss_time_S32_05-10_den_29-10.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Ghi chú review" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'S32 5-10 đến 29-10'!$A$2:$R$99</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'S32 5-10 đến 29-10'!$A$2:$R$103</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1604" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1666" uniqueCount="267">
   <si>
     <t xml:space="preserve">LOSS TIME MÃ S32 (OTHER SUPPORT OF PRODUCTION) - 05/10 ĐẾN 29/10/2026 - LÀM RIÊNG, KHÔNG LẪN MÃ KHÁC</t>
   </si>
@@ -459,6 +459,42 @@
   </si>
   <si>
     <t xml:space="preserve">Charge to: Unassigned (file Ép nóng)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AT654</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INLAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hỗ trợ khu vực INLAY (RESIN) - 25 full set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code RS-17-3256. Giờ bắt đầu/kết thúc là giờ chọn để đủ số giờ công trong báo cáo (người làm báo cáo: làm lúc rảnh, giờ nào cũng được)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hình: INLAY (RESIN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AT655</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hỗ trợ khu vực INLAY (RESIN) - 25 sét đuôi + hồng 3 đầu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code RS-17-3257. Giờ bắt đầu/kết thúc là giờ chọn để đủ số giờ công trong báo cáo (người làm báo cáo: làm lúc rảnh, giờ nào cũng được)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hỗ trợ khu vực INLAY (RESIN) - 25 full sét</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AT384</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hỗ trợ khu vực INLAY (RESIN) - 25 set hồng + 8 sét hộc kéo cửa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code RS-17-3080. Giờ bắt đầu/kết thúc là giờ chọn để đủ số giờ công trong báo cáo (người làm báo cáo: làm lúc rảnh, giờ nào cũng được)</t>
   </si>
   <si>
     <t xml:space="preserve">HS5913F1360</t>
@@ -1485,7 +1521,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R102"/>
+  <dimension ref="A1:R106"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -6361,132 +6397,134 @@
         <v>26</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="3" t="str">
+    <row r="94" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="13" t="str">
         <f aca="false">"W"&amp;WEEKNUM(B94,21)</f>
         <v>W44</v>
       </c>
-      <c r="B94" s="4" t="n">
-        <v>46323</v>
-      </c>
-      <c r="C94" s="5" t="s">
+      <c r="B94" s="14" t="n">
+        <v>46321</v>
+      </c>
+      <c r="C94" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="D94" s="3"/>
-      <c r="E94" s="3" t="n">
-        <v>47</v>
-      </c>
-      <c r="F94" s="3"/>
-      <c r="G94" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H94" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I94" s="5" t="s">
+      <c r="D94" s="13"/>
+      <c r="E94" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="F94" s="13"/>
+      <c r="G94" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="H94" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="I94" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="J94" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="K94" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="L94" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="M94" s="6" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="N94" s="6" t="n">
-        <v>0.756944444444444</v>
-      </c>
-      <c r="O94" s="7" t="n">
+      <c r="J94" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="K94" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="L94" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="M94" s="16" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="N94" s="16" t="n">
+        <v>0.520833333333333</v>
+      </c>
+      <c r="O94" s="17" t="n">
         <f aca="false">(N94-M94)*24</f>
-        <v>0.166666666666667</v>
-      </c>
-      <c r="P94" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q94" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="P94" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q94" s="17" t="n">
         <f aca="false">P94*O94</f>
-        <v>0.5</v>
-      </c>
-      <c r="R94" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="3" t="str">
+        <v>25</v>
+      </c>
+      <c r="R94" s="13" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="13" t="str">
         <f aca="false">"W"&amp;WEEKNUM(B95,21)</f>
         <v>W44</v>
       </c>
-      <c r="B95" s="4" t="n">
-        <v>46323</v>
-      </c>
-      <c r="C95" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="D95" s="3"/>
-      <c r="E95" s="3" t="n">
-        <v>188</v>
-      </c>
-      <c r="F95" s="3"/>
-      <c r="G95" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H95" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I95" s="5" t="s">
+      <c r="B95" s="14" t="n">
+        <v>46321</v>
+      </c>
+      <c r="C95" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D95" s="13"/>
+      <c r="E95" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="F95" s="13"/>
+      <c r="G95" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="H95" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="I95" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="J95" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="K95" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="L95" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="M95" s="6" t="n">
-        <v>0.7625</v>
-      </c>
-      <c r="N95" s="6" t="n">
-        <v>0.791666666666667</v>
-      </c>
-      <c r="O95" s="7" t="n">
+      <c r="J95" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="K95" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="L95" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="M95" s="16" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="N95" s="16" t="n">
+        <v>0.479166666666667</v>
+      </c>
+      <c r="O95" s="17" t="n">
         <f aca="false">(N95-M95)*24</f>
-        <v>0.7</v>
-      </c>
-      <c r="P95" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q95" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="P95" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q95" s="17" t="n">
         <f aca="false">P95*O95</f>
-        <v>2.1</v>
-      </c>
-      <c r="R95" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>20</v>
+      </c>
+      <c r="R95" s="13" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="13" t="str">
         <f aca="false">"W"&amp;WEEKNUM(B96,21)</f>
         <v>W44</v>
       </c>
       <c r="B96" s="14" t="n">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="C96" s="15" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D96" s="13"/>
-      <c r="E96" s="13"/>
+      <c r="E96" s="13" t="n">
+        <v>25</v>
+      </c>
       <c r="F96" s="13"/>
       <c r="G96" s="13" t="s">
-        <v>75</v>
+        <v>144</v>
       </c>
       <c r="H96" s="13" t="s">
         <v>21</v>
@@ -6495,88 +6533,88 @@
         <v>22</v>
       </c>
       <c r="J96" s="13" t="s">
-        <v>76</v>
+        <v>23</v>
       </c>
       <c r="K96" s="15" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="L96" s="15" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="M96" s="16" t="n">
-        <v>0.645833333333333</v>
+        <v>0.3125</v>
       </c>
       <c r="N96" s="16" t="n">
-        <v>0.8125</v>
+        <v>0.520833333333333</v>
       </c>
       <c r="O96" s="17" t="n">
         <f aca="false">(N96-M96)*24</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P96" s="13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q96" s="17" t="n">
         <f aca="false">P96*O96</f>
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="R96" s="13" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="3" t="str">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="13" t="str">
         <f aca="false">"W"&amp;WEEKNUM(B97,21)</f>
         <v>W44</v>
       </c>
-      <c r="B97" s="4" t="n">
-        <v>46324</v>
-      </c>
-      <c r="C97" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D97" s="3"/>
-      <c r="E97" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="F97" s="3"/>
-      <c r="G97" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H97" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I97" s="5" t="s">
+      <c r="B97" s="14" t="n">
+        <v>46321</v>
+      </c>
+      <c r="C97" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="D97" s="13"/>
+      <c r="E97" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="F97" s="13"/>
+      <c r="G97" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="H97" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="I97" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="J97" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="K97" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="L97" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="M97" s="6" t="n">
-        <v>0.583333333333333</v>
-      </c>
-      <c r="N97" s="6" t="n">
-        <v>0.586111111111111</v>
-      </c>
-      <c r="O97" s="7" t="n">
+      <c r="J97" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="K97" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="L97" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="M97" s="16" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="N97" s="16" t="n">
+        <v>0.429166666666667</v>
+      </c>
+      <c r="O97" s="17" t="n">
         <f aca="false">(N97-M97)*24</f>
-        <v>0.0666666666666667</v>
-      </c>
-      <c r="P97" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q97" s="7" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="P97" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q97" s="17" t="n">
         <f aca="false">P97*O97</f>
-        <v>0.2</v>
-      </c>
-      <c r="R97" s="3" t="s">
-        <v>41</v>
+        <v>14</v>
+      </c>
+      <c r="R97" s="13" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6585,14 +6623,14 @@
         <v>W44</v>
       </c>
       <c r="B98" s="4" t="n">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D98" s="3"/>
       <c r="E98" s="3" t="n">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="F98" s="3"/>
       <c r="G98" s="3" t="s">
@@ -6605,30 +6643,30 @@
         <v>22</v>
       </c>
       <c r="J98" s="3" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="K98" s="5" t="s">
-        <v>49</v>
+        <v>156</v>
       </c>
       <c r="L98" s="5" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="M98" s="6" t="n">
-        <v>0.586111111111111</v>
+        <v>0.75</v>
       </c>
       <c r="N98" s="6" t="n">
-        <v>0.588888888888889</v>
+        <v>0.756944444444444</v>
       </c>
       <c r="O98" s="7" t="n">
         <f aca="false">(N98-M98)*24</f>
-        <v>0.0666666666666667</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="P98" s="3" t="n">
         <v>3</v>
       </c>
       <c r="Q98" s="7" t="n">
         <f aca="false">P98*O98</f>
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="R98" s="3" t="s">
         <v>41</v>
@@ -6640,14 +6678,14 @@
         <v>W44</v>
       </c>
       <c r="B99" s="4" t="n">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D99" s="3"/>
       <c r="E99" s="3" t="n">
-        <v>26</v>
+        <v>188</v>
       </c>
       <c r="F99" s="3"/>
       <c r="G99" s="3" t="s">
@@ -6660,51 +6698,269 @@
         <v>22</v>
       </c>
       <c r="J99" s="3" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="K99" s="5" t="s">
-        <v>49</v>
+        <v>157</v>
       </c>
       <c r="L99" s="5" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="M99" s="6" t="n">
-        <v>0.588888888888889</v>
+        <v>0.7625</v>
       </c>
       <c r="N99" s="6" t="n">
-        <v>0.591666666666667</v>
+        <v>0.791666666666667</v>
       </c>
       <c r="O99" s="7" t="n">
         <f aca="false">(N99-M99)*24</f>
-        <v>0.0666666666666667</v>
+        <v>0.7</v>
       </c>
       <c r="P99" s="3" t="n">
         <v>3</v>
       </c>
       <c r="Q99" s="7" t="n">
         <f aca="false">P99*O99</f>
-        <v>0.2</v>
+        <v>2.1</v>
       </c>
       <c r="R99" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="P100" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="Q100" s="19" t="n">
-        <f aca="false">SUM(Q3:Q99)</f>
-        <v>4343.63333333333</v>
+    <row r="100" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="13" t="str">
+        <f aca="false">"W"&amp;WEEKNUM(B100,21)</f>
+        <v>W44</v>
+      </c>
+      <c r="B100" s="14" t="n">
+        <v>46323</v>
+      </c>
+      <c r="C100" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="D100" s="13"/>
+      <c r="E100" s="13"/>
+      <c r="F100" s="13"/>
+      <c r="G100" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="H100" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="I100" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="J100" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="K100" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="L100" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="M100" s="16" t="n">
+        <v>0.645833333333333</v>
+      </c>
+      <c r="N100" s="16" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="O100" s="17" t="n">
+        <f aca="false">(N100-M100)*24</f>
+        <v>4</v>
+      </c>
+      <c r="P100" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q100" s="17" t="n">
+        <f aca="false">P100*O100</f>
+        <v>12</v>
+      </c>
+      <c r="R100" s="13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="3" t="str">
+        <f aca="false">"W"&amp;WEEKNUM(B101,21)</f>
+        <v>W44</v>
+      </c>
+      <c r="B101" s="4" t="n">
+        <v>46324</v>
+      </c>
+      <c r="C101" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="D101" s="3"/>
+      <c r="E101" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="F101" s="3"/>
+      <c r="G101" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H101" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I101" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J101" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K101" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="L101" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M101" s="6" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="N101" s="6" t="n">
+        <v>0.586111111111111</v>
+      </c>
+      <c r="O101" s="7" t="n">
+        <f aca="false">(N101-M101)*24</f>
+        <v>0.0666666666666667</v>
+      </c>
+      <c r="P101" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q101" s="7" t="n">
+        <f aca="false">P101*O101</f>
+        <v>0.2</v>
+      </c>
+      <c r="R101" s="3" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="20" t="s">
-        <v>154</v>
+      <c r="A102" s="3" t="str">
+        <f aca="false">"W"&amp;WEEKNUM(B102,21)</f>
+        <v>W44</v>
+      </c>
+      <c r="B102" s="4" t="n">
+        <v>46324</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D102" s="3"/>
+      <c r="E102" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="F102" s="3"/>
+      <c r="G102" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H102" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I102" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J102" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K102" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="L102" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M102" s="6" t="n">
+        <v>0.586111111111111</v>
+      </c>
+      <c r="N102" s="6" t="n">
+        <v>0.588888888888889</v>
+      </c>
+      <c r="O102" s="7" t="n">
+        <f aca="false">(N102-M102)*24</f>
+        <v>0.0666666666666667</v>
+      </c>
+      <c r="P102" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q102" s="7" t="n">
+        <f aca="false">P102*O102</f>
+        <v>0.2</v>
+      </c>
+      <c r="R102" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="3" t="str">
+        <f aca="false">"W"&amp;WEEKNUM(B103,21)</f>
+        <v>W44</v>
+      </c>
+      <c r="B103" s="4" t="n">
+        <v>46324</v>
+      </c>
+      <c r="C103" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D103" s="3"/>
+      <c r="E103" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="F103" s="3"/>
+      <c r="G103" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H103" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I103" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J103" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K103" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="L103" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M103" s="6" t="n">
+        <v>0.588888888888889</v>
+      </c>
+      <c r="N103" s="6" t="n">
+        <v>0.591666666666667</v>
+      </c>
+      <c r="O103" s="7" t="n">
+        <f aca="false">(N103-M103)*24</f>
+        <v>0.0666666666666667</v>
+      </c>
+      <c r="P103" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q103" s="7" t="n">
+        <f aca="false">P103*O103</f>
+        <v>0.2</v>
+      </c>
+      <c r="R103" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P104" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q104" s="19" t="n">
+        <f aca="false">SUM(Q3:Q103)</f>
+        <v>4427.63333333333</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="20" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:R99"/>
+  <autoFilter ref="A2:R103"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -6721,29 +6977,29 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="4" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>26</v>
@@ -6773,7 +7029,10 @@
         <v>85</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>159</v>
+        <v>147</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6781,50 +7040,54 @@
         <v>46300</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="C4" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A4,21)</f>
         <v>W41</v>
       </c>
       <c r="D4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A4,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A4,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>46</v>
       </c>
       <c r="E4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A4,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A4,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>120</v>
       </c>
       <c r="F4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A4,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A4,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A4,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A4,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A4,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A4,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A4,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A4,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A4,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A4,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>0</v>
       </c>
       <c r="K4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A4,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A4,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L4" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A4,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M4" s="24" t="n">
-        <f aca="false">SUM(D4:L4)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A4,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A4,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N4" s="24" t="n">
+        <f aca="false">SUM(D4:M4)</f>
         <v>166</v>
       </c>
     </row>
@@ -6833,50 +7096,54 @@
         <v>46301</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="C5" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A5,21)</f>
         <v>W41</v>
       </c>
       <c r="D5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A5,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A5,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>55</v>
       </c>
       <c r="E5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A5,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A5,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>120</v>
       </c>
       <c r="F5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A5,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A5,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A5,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A5,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A5,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A5,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A5,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A5,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A5,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A5,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>0</v>
       </c>
       <c r="K5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A5,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A5,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L5" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A5,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M5" s="24" t="n">
-        <f aca="false">SUM(D5:L5)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A5,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A5,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N5" s="24" t="n">
+        <f aca="false">SUM(D5:M5)</f>
         <v>175</v>
       </c>
     </row>
@@ -6885,50 +7152,54 @@
         <v>46302</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="C6" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A6,21)</f>
         <v>W41</v>
       </c>
       <c r="D6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A6,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A6,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A6,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A6,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>112</v>
       </c>
       <c r="F6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A6,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A6,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A6,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A6,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A6,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A6,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A6,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A6,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A6,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A6,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>0</v>
       </c>
       <c r="K6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A6,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A6,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L6" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A6,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M6" s="24" t="n">
-        <f aca="false">SUM(D6:L6)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A6,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A6,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N6" s="24" t="n">
+        <f aca="false">SUM(D6:M6)</f>
         <v>112</v>
       </c>
     </row>
@@ -6937,50 +7208,54 @@
         <v>46303</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="C7" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A7,21)</f>
         <v>W41</v>
       </c>
       <c r="D7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A7,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A7,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A7,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A7,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>104</v>
       </c>
       <c r="F7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A7,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A7,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0.2</v>
       </c>
       <c r="G7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A7,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A7,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A7,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A7,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A7,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A7,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A7,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A7,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>0</v>
       </c>
       <c r="K7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A7,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A7,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L7" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A7,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M7" s="24" t="n">
-        <f aca="false">SUM(D7:L7)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A7,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A7,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N7" s="24" t="n">
+        <f aca="false">SUM(D7:M7)</f>
         <v>104.2</v>
       </c>
     </row>
@@ -6989,50 +7264,54 @@
         <v>46304</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C8" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A8,21)</f>
         <v>W41</v>
       </c>
       <c r="D8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A8,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A8,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A8,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A8,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>132</v>
       </c>
       <c r="F8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A8,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A8,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0.6</v>
       </c>
       <c r="G8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A8,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A8,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A8,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A8,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A8,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A8,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A8,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A8,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>0</v>
       </c>
       <c r="K8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A8,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A8,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L8" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A8,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M8" s="24" t="n">
-        <f aca="false">SUM(D8:L8)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A8,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A8,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N8" s="24" t="n">
+        <f aca="false">SUM(D8:M8)</f>
         <v>132.6</v>
       </c>
     </row>
@@ -7041,50 +7320,54 @@
         <v>46305</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="C9" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A9,21)</f>
         <v>W41</v>
       </c>
       <c r="D9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A9,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A9,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A9,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A9,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>116</v>
       </c>
       <c r="F9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A9,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A9,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A9,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A9,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>3</v>
       </c>
       <c r="H9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A9,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A9,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A9,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A9,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A9,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A9,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>0</v>
       </c>
       <c r="K9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A9,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A9,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L9" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A9,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M9" s="24" t="n">
-        <f aca="false">SUM(D9:L9)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A9,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A9,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N9" s="24" t="n">
+        <f aca="false">SUM(D9:M9)</f>
         <v>119</v>
       </c>
     </row>
@@ -7093,50 +7376,54 @@
         <v>46306</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="C10" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A10,21)</f>
         <v>W41</v>
       </c>
       <c r="D10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A10,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A10,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A10,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A10,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>72</v>
       </c>
       <c r="F10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A10,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A10,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A10,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A10,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A10,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A10,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A10,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A10,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A10,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A10,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>0</v>
       </c>
       <c r="K10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A10,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A10,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L10" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A10,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M10" s="24" t="n">
-        <f aca="false">SUM(D10:L10)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A10,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A10,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N10" s="24" t="n">
+        <f aca="false">SUM(D10:M10)</f>
         <v>72</v>
       </c>
     </row>
@@ -7145,50 +7432,54 @@
         <v>46307</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="C11" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A11,21)</f>
         <v>W42</v>
       </c>
       <c r="D11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A11,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A11,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A11,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A11,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>132</v>
       </c>
       <c r="F11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A11,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A11,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A11,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A11,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A11,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A11,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A11,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A11,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>18</v>
       </c>
       <c r="J11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A11,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A11,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>144</v>
       </c>
       <c r="K11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A11,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A11,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L11" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A11,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M11" s="24" t="n">
-        <f aca="false">SUM(D11:L11)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A11,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A11,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N11" s="24" t="n">
+        <f aca="false">SUM(D11:M11)</f>
         <v>294</v>
       </c>
     </row>
@@ -7197,50 +7488,54 @@
         <v>46308</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="C12" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A12,21)</f>
         <v>W42</v>
       </c>
       <c r="D12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A12,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A12,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A12,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A12,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>140</v>
       </c>
       <c r="F12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A12,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A12,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A12,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A12,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A12,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A12,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A12,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A12,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>4.5</v>
       </c>
       <c r="J12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A12,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A12,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>144</v>
       </c>
       <c r="K12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A12,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A12,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L12" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A12,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M12" s="24" t="n">
-        <f aca="false">SUM(D12:L12)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A12,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M12" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A12,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N12" s="24" t="n">
+        <f aca="false">SUM(D12:M12)</f>
         <v>288.5</v>
       </c>
     </row>
@@ -7249,50 +7544,54 @@
         <v>46309</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="C13" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A13,21)</f>
         <v>W42</v>
       </c>
       <c r="D13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A13,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A13,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A13,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A13,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>132</v>
       </c>
       <c r="F13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A13,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A13,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A13,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A13,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A13,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A13,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>2</v>
       </c>
       <c r="I13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A13,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A13,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A13,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A13,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>144</v>
       </c>
       <c r="K13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A13,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A13,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L13" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A13,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M13" s="24" t="n">
-        <f aca="false">SUM(D13:L13)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A13,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A13,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N13" s="24" t="n">
+        <f aca="false">SUM(D13:M13)</f>
         <v>278</v>
       </c>
     </row>
@@ -7301,50 +7600,54 @@
         <v>46310</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="C14" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A14,21)</f>
         <v>W42</v>
       </c>
       <c r="D14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A14,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A14,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A14,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A14,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>132</v>
       </c>
       <c r="F14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A14,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A14,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A14,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A14,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0.333333333333333</v>
       </c>
       <c r="H14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A14,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A14,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A14,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A14,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A14,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A14,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>144</v>
       </c>
       <c r="K14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A14,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A14,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L14" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A14,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A14,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
         <v>32</v>
       </c>
-      <c r="M14" s="24" t="n">
-        <f aca="false">SUM(D14:L14)</f>
+      <c r="M14" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A14,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N14" s="24" t="n">
+        <f aca="false">SUM(D14:M14)</f>
         <v>308.333333333333</v>
       </c>
     </row>
@@ -7353,50 +7656,54 @@
         <v>46311</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C15" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A15,21)</f>
         <v>W42</v>
       </c>
       <c r="D15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A15,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A15,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A15,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A15,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>116</v>
       </c>
       <c r="F15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A15,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A15,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0.75</v>
       </c>
       <c r="G15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A15,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A15,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A15,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A15,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A15,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A15,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A15,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A15,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>144</v>
       </c>
       <c r="K15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A15,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A15,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>9</v>
       </c>
       <c r="L15" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A15,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="24" t="n">
-        <f aca="false">SUM(D15:L15)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A15,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M15" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A15,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N15" s="24" t="n">
+        <f aca="false">SUM(D15:M15)</f>
         <v>269.75</v>
       </c>
     </row>
@@ -7405,50 +7712,54 @@
         <v>46312</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="C16" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A16,21)</f>
         <v>W42</v>
       </c>
       <c r="D16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A16,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A16,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A16,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A16,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>128</v>
       </c>
       <c r="F16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A16,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A16,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0.2</v>
       </c>
       <c r="G16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A16,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A16,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A16,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A16,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A16,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A16,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A16,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A16,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>96</v>
       </c>
       <c r="K16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A16,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A16,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L16" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A16,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M16" s="24" t="n">
-        <f aca="false">SUM(D16:L16)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A16,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M16" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A16,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N16" s="24" t="n">
+        <f aca="false">SUM(D16:M16)</f>
         <v>224.2</v>
       </c>
     </row>
@@ -7457,50 +7768,54 @@
         <v>46314</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="C17" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A17,21)</f>
         <v>W43</v>
       </c>
       <c r="D17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A17,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A17,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A17,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A17,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>136</v>
       </c>
       <c r="F17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A17,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A17,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0.35</v>
       </c>
       <c r="G17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A17,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A17,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A17,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A17,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A17,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A17,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A17,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A17,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>144</v>
       </c>
       <c r="K17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A17,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A17,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L17" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A17,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M17" s="24" t="n">
-        <f aca="false">SUM(D17:L17)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A17,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M17" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A17,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N17" s="24" t="n">
+        <f aca="false">SUM(D17:M17)</f>
         <v>280.35</v>
       </c>
     </row>
@@ -7509,50 +7824,54 @@
         <v>46315</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="C18" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A18,21)</f>
         <v>W43</v>
       </c>
       <c r="D18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A18,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A18,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A18,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A18,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>136</v>
       </c>
       <c r="F18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A18,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A18,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0.4</v>
       </c>
       <c r="G18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A18,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A18,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>4</v>
       </c>
       <c r="H18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A18,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A18,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A18,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A18,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A18,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A18,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>144</v>
       </c>
       <c r="K18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A18,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A18,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>24</v>
       </c>
       <c r="L18" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A18,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M18" s="24" t="n">
-        <f aca="false">SUM(D18:L18)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A18,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M18" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A18,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N18" s="24" t="n">
+        <f aca="false">SUM(D18:M18)</f>
         <v>308.4</v>
       </c>
     </row>
@@ -7561,50 +7880,54 @@
         <v>46316</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="C19" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A19,21)</f>
         <v>W43</v>
       </c>
       <c r="D19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A19,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A19,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A19,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A19,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>128</v>
       </c>
       <c r="F19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A19,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A19,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A19,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A19,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A19,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A19,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A19,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A19,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A19,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A19,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>144</v>
       </c>
       <c r="K19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A19,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A19,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L19" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A19,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M19" s="24" t="n">
-        <f aca="false">SUM(D19:L19)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A19,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M19" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A19,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N19" s="24" t="n">
+        <f aca="false">SUM(D19:M19)</f>
         <v>272</v>
       </c>
     </row>
@@ -7613,50 +7936,54 @@
         <v>46317</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="C20" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A20,21)</f>
         <v>W43</v>
       </c>
       <c r="D20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A20,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A20,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A20,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A20,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>108</v>
       </c>
       <c r="F20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A20,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A20,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>3.1</v>
       </c>
       <c r="G20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A20,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A20,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A20,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A20,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A20,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A20,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A20,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A20,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>144</v>
       </c>
       <c r="K20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A20,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A20,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L20" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A20,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M20" s="24" t="n">
-        <f aca="false">SUM(D20:L20)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A20,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M20" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A20,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N20" s="24" t="n">
+        <f aca="false">SUM(D20:M20)</f>
         <v>255.1</v>
       </c>
     </row>
@@ -7665,50 +7992,54 @@
         <v>46318</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C21" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A21,21)</f>
         <v>W43</v>
       </c>
       <c r="D21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A21,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A21,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A21,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A21,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>128</v>
       </c>
       <c r="F21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A21,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A21,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A21,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A21,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>48</v>
       </c>
       <c r="H21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A21,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A21,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>3.6</v>
       </c>
       <c r="I21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A21,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A21,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A21,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A21,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>144</v>
       </c>
       <c r="K21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A21,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A21,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L21" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A21,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M21" s="24" t="n">
-        <f aca="false">SUM(D21:L21)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A21,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M21" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A21,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N21" s="24" t="n">
+        <f aca="false">SUM(D21:M21)</f>
         <v>323.6</v>
       </c>
     </row>
@@ -7717,50 +8048,54 @@
         <v>46319</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="C22" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A22,21)</f>
         <v>W43</v>
       </c>
       <c r="D22" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A22,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A22,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E22" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A22,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A22,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>88</v>
       </c>
       <c r="F22" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A22,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A22,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0.4</v>
       </c>
       <c r="G22" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A22,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A22,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>17</v>
       </c>
       <c r="H22" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A22,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A22,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I22" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A22,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A22,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J22" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A22,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A22,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>96</v>
       </c>
       <c r="K22" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A22,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A22,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>16</v>
       </c>
       <c r="L22" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A22,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A22,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
         <v>24</v>
       </c>
-      <c r="M22" s="24" t="n">
-        <f aca="false">SUM(D22:L22)</f>
+      <c r="M22" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A22,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N22" s="24" t="n">
+        <f aca="false">SUM(D22:M22)</f>
         <v>241.4</v>
       </c>
     </row>
@@ -7769,50 +8104,54 @@
         <v>46320</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="C23" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A23,21)</f>
         <v>W43</v>
       </c>
       <c r="D23" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A23,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A23,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E23" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A23,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A23,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>0</v>
       </c>
       <c r="F23" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A23,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A23,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G23" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A23,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A23,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H23" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A23,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A23,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I23" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A23,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A23,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J23" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A23,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A23,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>96</v>
       </c>
       <c r="K23" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A23,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A23,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>6</v>
       </c>
       <c r="L23" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A23,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M23" s="24" t="n">
-        <f aca="false">SUM(D23:L23)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A23,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M23" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A23,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N23" s="24" t="n">
+        <f aca="false">SUM(D23:M23)</f>
         <v>102</v>
       </c>
     </row>
@@ -7821,51 +8160,55 @@
         <v>46321</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="C24" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A24,21)</f>
         <v>W44</v>
       </c>
       <c r="D24" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A24,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A24,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>2</v>
       </c>
       <c r="E24" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A24,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A24,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>0</v>
       </c>
       <c r="F24" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A24,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A24,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0</v>
       </c>
       <c r="G24" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A24,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A24,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H24" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A24,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A24,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I24" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A24,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A24,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J24" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A24,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A24,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>0</v>
       </c>
       <c r="K24" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A24,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A24,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L24" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A24,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M24" s="24" t="n">
-        <f aca="false">SUM(D24:L24)</f>
-        <v>2</v>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A24,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M24" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A24,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>84</v>
+      </c>
+      <c r="N24" s="24" t="n">
+        <f aca="false">SUM(D24:M24)</f>
+        <v>86</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7873,50 +8216,54 @@
         <v>46323</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="C25" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A25,21)</f>
         <v>W44</v>
       </c>
       <c r="D25" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A25,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A25,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E25" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A25,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A25,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>0</v>
       </c>
       <c r="F25" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A25,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A25,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>2.6</v>
       </c>
       <c r="G25" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A25,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A25,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H25" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A25,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A25,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>12</v>
       </c>
       <c r="I25" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A25,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A25,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J25" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A25,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A25,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>0</v>
       </c>
       <c r="K25" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A25,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A25,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L25" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A25,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M25" s="24" t="n">
-        <f aca="false">SUM(D25:L25)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A25,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M25" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A25,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N25" s="24" t="n">
+        <f aca="false">SUM(D25:M25)</f>
         <v>14.6</v>
       </c>
     </row>
@@ -7925,56 +8272,60 @@
         <v>46324</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="C26" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A26,21)</f>
         <v>W44</v>
       </c>
       <c r="D26" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A26,'S32 5-10 đến 29-10'!$R$3:$R$99,D$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A26,'S32 5-10 đến 29-10'!$R$3:$R$103,D$3)</f>
         <v>0</v>
       </c>
       <c r="E26" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A26,'S32 5-10 đến 29-10'!$R$3:$R$99,E$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A26,'S32 5-10 đến 29-10'!$R$3:$R$103,E$3)</f>
         <v>0</v>
       </c>
       <c r="F26" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A26,'S32 5-10 đến 29-10'!$R$3:$R$99,F$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A26,'S32 5-10 đến 29-10'!$R$3:$R$103,F$3)</f>
         <v>0.6</v>
       </c>
       <c r="G26" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A26,'S32 5-10 đến 29-10'!$R$3:$R$99,G$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A26,'S32 5-10 đến 29-10'!$R$3:$R$103,G$3)</f>
         <v>0</v>
       </c>
       <c r="H26" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A26,'S32 5-10 đến 29-10'!$R$3:$R$99,H$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A26,'S32 5-10 đến 29-10'!$R$3:$R$103,H$3)</f>
         <v>0</v>
       </c>
       <c r="I26" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A26,'S32 5-10 đến 29-10'!$R$3:$R$99,I$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A26,'S32 5-10 đến 29-10'!$R$3:$R$103,I$3)</f>
         <v>0</v>
       </c>
       <c r="J26" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A26,'S32 5-10 đến 29-10'!$R$3:$R$99,J$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A26,'S32 5-10 đến 29-10'!$R$3:$R$103,J$3)</f>
         <v>0</v>
       </c>
       <c r="K26" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A26,'S32 5-10 đến 29-10'!$R$3:$R$99,K$3)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A26,'S32 5-10 đến 29-10'!$R$3:$R$103,K$3)</f>
         <v>0</v>
       </c>
       <c r="L26" s="23" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$B$3:$B$99,$A26,'S32 5-10 đến 29-10'!$R$3:$R$99,L$3)</f>
-        <v>0</v>
-      </c>
-      <c r="M26" s="24" t="n">
-        <f aca="false">SUM(D26:L26)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A26,'S32 5-10 đến 29-10'!$R$3:$R$103,L$3)</f>
+        <v>0</v>
+      </c>
+      <c r="M26" s="23" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$B$3:$B$103,$A26,'S32 5-10 đến 29-10'!$R$3:$R$103,M$3)</f>
+        <v>0</v>
+      </c>
+      <c r="N26" s="24" t="n">
+        <f aca="false">SUM(D26:M26)</f>
         <v>0.6</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="25" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
@@ -8016,56 +8367,60 @@
       </c>
       <c r="M27" s="24" t="n">
         <f aca="false">SUM(M4:M26)</f>
-        <v>4343.63333333333</v>
+        <v>84</v>
+      </c>
+      <c r="N27" s="24" t="n">
+        <f aca="false">SUM(N4:N26)</f>
+        <v>4427.63333333333</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="18" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="26" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="B31" s="27" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$A$3:$A$99,A31)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$A$3:$A$103,A31)</f>
         <v>880.8</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="26" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="B32" s="27" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$A$3:$A$99,A32)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$A$3:$A$103,A32)</f>
         <v>1662.78333333333</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="26" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="B33" s="27" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$A$3:$A$99,A33)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$A$3:$A$103,A33)</f>
         <v>1782.85</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="26" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="B34" s="27" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$A$3:$A$99,A34)</f>
-        <v>17.2</v>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$A$3:$A$103,A34)</f>
+        <v>101.2</v>
       </c>
     </row>
   </sheetData>
@@ -8084,7 +8439,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -8102,19 +8457,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>13</v>
@@ -8123,19 +8478,19 @@
         <v>14</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="I1" s="28" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="J1" s="28" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="K1" s="28" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="L1" s="28" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11384,189 +11739,191 @@
         <v>26</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="29" t="n">
-        <v>46323</v>
-      </c>
-      <c r="B93" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="C93" s="31" t="s">
+    <row r="93" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="40" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B93" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C93" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="D93" s="41" t="s">
         <v>144</v>
       </c>
-      <c r="D93" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="E93" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="F93" s="32" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G93" s="32" t="n">
-        <v>0.756944444444444</v>
-      </c>
-      <c r="H93" s="30" t="n">
-        <v>3</v>
+      <c r="E93" s="41" t="s">
+        <v>23</v>
+      </c>
+      <c r="F93" s="43" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="G93" s="43" t="n">
+        <v>0.520833333333333</v>
+      </c>
+      <c r="H93" s="41" t="n">
+        <v>5</v>
       </c>
       <c r="I93" s="33" t="s">
         <v>143</v>
       </c>
       <c r="J93" s="34" t="n">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="K93" s="35" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="L93" s="34" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="29" t="n">
-        <v>46323</v>
-      </c>
-      <c r="B94" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="C94" s="31" t="s">
-        <v>145</v>
-      </c>
-      <c r="D94" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="E94" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="F94" s="32" t="n">
-        <v>0.7625</v>
-      </c>
-      <c r="G94" s="32" t="n">
-        <v>0.791666666666667</v>
-      </c>
-      <c r="H94" s="30" t="n">
-        <v>3</v>
+        <v>147</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="40" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B94" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C94" s="42" t="s">
+        <v>149</v>
+      </c>
+      <c r="D94" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="E94" s="41" t="s">
+        <v>23</v>
+      </c>
+      <c r="F94" s="43" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="G94" s="43" t="n">
+        <v>0.479166666666667</v>
+      </c>
+      <c r="H94" s="41" t="n">
+        <v>5</v>
       </c>
       <c r="I94" s="33" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J94" s="34" t="n">
-        <v>188</v>
+        <v>25</v>
       </c>
       <c r="K94" s="35" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="L94" s="34" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="40" t="n">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="B95" s="41" t="s">
         <v>21</v>
       </c>
       <c r="C95" s="42" t="s">
+        <v>151</v>
+      </c>
+      <c r="D95" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="E95" s="41" t="s">
+        <v>23</v>
+      </c>
+      <c r="F95" s="43" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="G95" s="43" t="n">
+        <v>0.520833333333333</v>
+      </c>
+      <c r="H95" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="I95" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="J95" s="34" t="n">
+        <v>25</v>
+      </c>
+      <c r="K95" s="35" t="s">
+        <v>150</v>
+      </c>
+      <c r="L95" s="34" t="s">
         <v>147</v>
       </c>
-      <c r="D95" s="41" t="s">
-        <v>75</v>
-      </c>
-      <c r="E95" s="41" t="s">
-        <v>76</v>
-      </c>
-      <c r="F95" s="43" t="n">
-        <v>0.645833333333333</v>
-      </c>
-      <c r="G95" s="43" t="n">
-        <v>0.8125</v>
-      </c>
-      <c r="H95" s="41" t="n">
-        <v>3</v>
-      </c>
-      <c r="I95" s="33" t="s">
-        <v>146</v>
-      </c>
-      <c r="J95" s="34"/>
-      <c r="K95" s="35" t="s">
-        <v>148</v>
-      </c>
-      <c r="L95" s="34" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="29" t="n">
-        <v>46324</v>
-      </c>
-      <c r="B96" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="C96" s="31" t="s">
-        <v>49</v>
-      </c>
-      <c r="D96" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="E96" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="F96" s="32" t="n">
-        <v>0.583333333333333</v>
-      </c>
-      <c r="G96" s="32" t="n">
-        <v>0.586111111111111</v>
-      </c>
-      <c r="H96" s="30" t="n">
-        <v>3</v>
+    </row>
+    <row r="96" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="40" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B96" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C96" s="42" t="s">
+        <v>153</v>
+      </c>
+      <c r="D96" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="E96" s="41" t="s">
+        <v>23</v>
+      </c>
+      <c r="F96" s="43" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="G96" s="43" t="n">
+        <v>0.429166666666667</v>
+      </c>
+      <c r="H96" s="41" t="n">
+        <v>5</v>
       </c>
       <c r="I96" s="33" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="J96" s="34" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K96" s="35" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="L96" s="34" t="s">
-        <v>41</v>
+        <v>147</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="29" t="n">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="B97" s="30" t="s">
         <v>21</v>
       </c>
       <c r="C97" s="31" t="s">
-        <v>49</v>
+        <v>156</v>
       </c>
       <c r="D97" s="30" t="s">
         <v>20</v>
       </c>
       <c r="E97" s="30" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="F97" s="32" t="n">
-        <v>0.586111111111111</v>
+        <v>0.75</v>
       </c>
       <c r="G97" s="32" t="n">
-        <v>0.588888888888889</v>
+        <v>0.756944444444444</v>
       </c>
       <c r="H97" s="30" t="n">
         <v>3</v>
       </c>
       <c r="I97" s="33" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="J97" s="34" t="n">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="K97" s="35" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="L97" s="34" t="s">
         <v>41</v>
@@ -11574,45 +11931,195 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="29" t="n">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="B98" s="30" t="s">
         <v>21</v>
       </c>
       <c r="C98" s="31" t="s">
-        <v>49</v>
+        <v>157</v>
       </c>
       <c r="D98" s="30" t="s">
         <v>20</v>
       </c>
       <c r="E98" s="30" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="F98" s="32" t="n">
-        <v>0.588888888888889</v>
+        <v>0.7625</v>
       </c>
       <c r="G98" s="32" t="n">
-        <v>0.591666666666667</v>
+        <v>0.791666666666667</v>
       </c>
       <c r="H98" s="30" t="n">
         <v>3</v>
       </c>
       <c r="I98" s="33" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="J98" s="34" t="n">
-        <v>26</v>
+        <v>188</v>
       </c>
       <c r="K98" s="35" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="L98" s="34" t="s">
         <v>41</v>
       </c>
     </row>
+    <row r="99" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="40" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B99" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C99" s="42" t="s">
+        <v>159</v>
+      </c>
+      <c r="D99" s="41" t="s">
+        <v>75</v>
+      </c>
+      <c r="E99" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="F99" s="43" t="n">
+        <v>0.645833333333333</v>
+      </c>
+      <c r="G99" s="43" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="H99" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="I99" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="J99" s="34"/>
+      <c r="K99" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="L99" s="34" t="s">
+        <v>79</v>
+      </c>
+    </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="20" t="s">
-        <v>183</v>
+      <c r="A100" s="29" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B100" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C100" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D100" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E100" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="F100" s="32" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="G100" s="32" t="n">
+        <v>0.586111111111111</v>
+      </c>
+      <c r="H100" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="I100" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="J100" s="34" t="n">
+        <v>26</v>
+      </c>
+      <c r="K100" s="35" t="s">
+        <v>162</v>
+      </c>
+      <c r="L100" s="34" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="29" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B101" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C101" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D101" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E101" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="F101" s="32" t="n">
+        <v>0.586111111111111</v>
+      </c>
+      <c r="G101" s="32" t="n">
+        <v>0.588888888888889</v>
+      </c>
+      <c r="H101" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="I101" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="J101" s="34" t="n">
+        <v>26</v>
+      </c>
+      <c r="K101" s="35" t="s">
+        <v>162</v>
+      </c>
+      <c r="L101" s="34" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="29" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B102" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C102" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D102" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E102" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="F102" s="32" t="n">
+        <v>0.588888888888889</v>
+      </c>
+      <c r="G102" s="32" t="n">
+        <v>0.591666666666667</v>
+      </c>
+      <c r="H102" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="I102" s="33" t="s">
+        <v>164</v>
+      </c>
+      <c r="J102" s="34" t="n">
+        <v>26</v>
+      </c>
+      <c r="K102" s="35" t="s">
+        <v>162</v>
+      </c>
+      <c r="L102" s="34" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="20" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -11631,7 +12138,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -11643,7 +12150,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11651,16 +12158,16 @@
         <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11671,7 +12178,7 @@
         <v>9.2</v>
       </c>
       <c r="C4" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$R$3:$R$99,A4)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$R$3:$R$103,A4)</f>
         <v>9.2</v>
       </c>
       <c r="D4" s="46" t="n">
@@ -11691,7 +12198,7 @@
         <v>2280</v>
       </c>
       <c r="C5" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$R$3:$R$99,A5)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$R$3:$R$103,A5)</f>
         <v>2280</v>
       </c>
       <c r="D5" s="46" t="n">
@@ -11711,7 +12218,7 @@
         <v>22.5</v>
       </c>
       <c r="C6" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$R$3:$R$99,A6)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$R$3:$R$103,A6)</f>
         <v>22.5</v>
       </c>
       <c r="D6" s="46" t="n">
@@ -11731,7 +12238,7 @@
         <v>103</v>
       </c>
       <c r="C7" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$R$3:$R$99,A7)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$R$3:$R$103,A7)</f>
         <v>103</v>
       </c>
       <c r="D7" s="46" t="n">
@@ -11751,7 +12258,7 @@
         <v>72.3333</v>
       </c>
       <c r="C8" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$R$3:$R$99,A8)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$R$3:$R$103,A8)</f>
         <v>72.3333333333333</v>
       </c>
       <c r="D8" s="46" t="n">
@@ -11771,7 +12278,7 @@
         <v>17.8333</v>
       </c>
       <c r="C9" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$R$3:$R$99,A9)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$R$3:$R$103,A9)</f>
         <v>17.6</v>
       </c>
       <c r="D9" s="46" t="n">
@@ -11791,7 +12298,7 @@
         <v>1728</v>
       </c>
       <c r="C10" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$R$3:$R$99,A10)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$R$3:$R$103,A10)</f>
         <v>1728</v>
       </c>
       <c r="D10" s="46" t="n">
@@ -11811,7 +12318,7 @@
         <v>55</v>
       </c>
       <c r="C11" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$R$3:$R$99,A11)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$R$3:$R$103,A11)</f>
         <v>55</v>
       </c>
       <c r="D11" s="46" t="n">
@@ -11831,7 +12338,7 @@
         <v>56</v>
       </c>
       <c r="C12" s="46" t="n">
-        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$99,'S32 5-10 đến 29-10'!$R$3:$R$99,A12)</f>
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$R$3:$R$103,A12)</f>
         <v>56</v>
       </c>
       <c r="D12" s="46" t="n">
@@ -11844,29 +12351,49 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="47" t="s">
-        <v>153</v>
-      </c>
-      <c r="B13" s="48" t="n">
-        <f aca="false">SUM(B4:B12)</f>
-        <v>4343.8666</v>
-      </c>
-      <c r="C13" s="48" t="n">
-        <f aca="false">SUM(C4:C12)</f>
-        <v>4343.63333333333</v>
-      </c>
-      <c r="D13" s="48" t="n">
-        <f aca="false">SUM(D4:D12)</f>
+      <c r="A13" s="44" t="s">
+        <v>147</v>
+      </c>
+      <c r="B13" s="45" t="n">
+        <v>84</v>
+      </c>
+      <c r="C13" s="46" t="n">
+        <f aca="false">SUMIFS('S32 5-10 đến 29-10'!$Q$3:$Q$103,'S32 5-10 đến 29-10'!$R$3:$R$103,A13)</f>
+        <v>84</v>
+      </c>
+      <c r="D13" s="46" t="n">
+        <f aca="false">C13-B13</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="3" t="str">
+        <f aca="false">IF(ABS(D13)&lt;0.01,"Khớp","Lệch")</f>
+        <v>Khớp</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="47" t="s">
+        <v>165</v>
+      </c>
+      <c r="B14" s="48" t="n">
+        <f aca="false">SUM(B4:B13)</f>
+        <v>4427.8666</v>
+      </c>
+      <c r="C14" s="48" t="n">
+        <f aca="false">SUM(C4:C13)</f>
+        <v>4427.63333333333</v>
+      </c>
+      <c r="D14" s="48" t="n">
+        <f aca="false">SUM(D4:D13)</f>
         <v>-0.233266666666665</v>
       </c>
-      <c r="E13" s="25" t="str">
-        <f aca="false">IF(ABS(D13)&lt;0.01,"Khớp","Lệch")</f>
+      <c r="E14" s="25" t="str">
+        <f aca="false">IF(ABS(D14)&lt;0.01,"Khớp","Lệch")</f>
         <v>Lệch</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
-        <v>189</v>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="20" t="s">
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -11897,19 +12424,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11920,10 +12447,10 @@
         <v>26</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="D2" s="26" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="E2" s="26" t="n">
         <v>10</v>
@@ -11937,10 +12464,10 @@
         <v>26</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="E3" s="26" t="n">
         <v>5</v>
@@ -11954,10 +12481,10 @@
         <v>26</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>10</v>
@@ -11971,10 +12498,10 @@
         <v>26</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="E5" s="26" t="n">
         <v>27</v>
@@ -11988,10 +12515,10 @@
         <v>26</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>23</v>
@@ -12005,10 +12532,10 @@
         <v>26</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="E7" s="26" t="n">
         <v>27</v>
@@ -12022,10 +12549,10 @@
         <v>26</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>23</v>
@@ -12039,10 +12566,10 @@
         <v>62</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="E9" s="26" t="n">
         <v>50</v>
@@ -12056,10 +12583,10 @@
         <v>62</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>100</v>
@@ -12073,10 +12600,10 @@
         <v>65</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E11" s="26" t="n">
         <v>13</v>
@@ -12090,10 +12617,10 @@
         <v>65</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>13</v>
@@ -12107,10 +12634,10 @@
         <v>65</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E13" s="26" t="n">
         <v>13</v>
@@ -12124,10 +12651,10 @@
         <v>65</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>13</v>
@@ -12141,10 +12668,10 @@
         <v>65</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E15" s="26" t="n">
         <v>13</v>
@@ -12158,10 +12685,10 @@
         <v>65</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>13</v>
@@ -12175,10 +12702,10 @@
         <v>65</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="D17" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E17" s="26" t="n">
         <v>13</v>
@@ -12192,10 +12719,10 @@
         <v>65</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="D18" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E18" s="26" t="n">
         <v>13</v>
@@ -12209,10 +12736,10 @@
         <v>65</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="D19" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E19" s="26" t="n">
         <v>13</v>
@@ -12226,10 +12753,10 @@
         <v>65</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="D20" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E20" s="26" t="n">
         <v>13</v>
@@ -12243,10 +12770,10 @@
         <v>65</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="D21" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E21" s="26" t="n">
         <v>13</v>
@@ -12260,10 +12787,10 @@
         <v>65</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="D22" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E22" s="26" t="n">
         <v>13</v>
@@ -12277,10 +12804,10 @@
         <v>65</v>
       </c>
       <c r="C23" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="D23" s="26" t="s">
         <v>217</v>
-      </c>
-      <c r="D23" s="26" t="s">
-        <v>205</v>
       </c>
       <c r="E23" s="26" t="n">
         <v>13</v>
@@ -12294,10 +12821,10 @@
         <v>65</v>
       </c>
       <c r="C24" s="26" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E24" s="26" t="n">
         <v>13</v>
@@ -12311,10 +12838,10 @@
         <v>65</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D25" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E25" s="26" t="n">
         <v>455</v>
@@ -12328,10 +12855,10 @@
         <v>65</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="D26" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E26" s="26" t="n">
         <v>299</v>
@@ -12345,10 +12872,10 @@
         <v>65</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="D27" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E27" s="26" t="n">
         <v>286</v>
@@ -12362,10 +12889,10 @@
         <v>65</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D28" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E28" s="26" t="n">
         <v>1092</v>
@@ -12379,10 +12906,10 @@
         <v>65</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="D29" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E29" s="26" t="n">
         <v>156</v>
@@ -12396,10 +12923,10 @@
         <v>65</v>
       </c>
       <c r="C30" s="26" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="D30" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E30" s="26" t="n">
         <v>13</v>
@@ -12413,10 +12940,10 @@
         <v>65</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="D31" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E31" s="26" t="n">
         <v>13</v>
@@ -12430,10 +12957,10 @@
         <v>65</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="D32" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E32" s="26" t="n">
         <v>13</v>
@@ -12447,10 +12974,10 @@
         <v>65</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="D33" s="26" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E33" s="26" t="n">
         <v>13</v>
@@ -12467,7 +12994,7 @@
         <v>74</v>
       </c>
       <c r="D34" s="26" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="E34" s="26" t="n">
         <v>100</v>
@@ -12484,7 +13011,7 @@
         <v>80</v>
       </c>
       <c r="D35" s="26" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="E35" s="26" t="n">
         <v>4</v>
@@ -12501,7 +13028,7 @@
         <v>109</v>
       </c>
       <c r="D36" s="26" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="E36" s="26" t="n">
         <v>30</v>
@@ -12518,7 +13045,7 @@
         <v>110</v>
       </c>
       <c r="D37" s="26" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="E37" s="26" t="n">
         <v>2</v>
@@ -12535,7 +13062,7 @@
         <v>114</v>
       </c>
       <c r="D38" s="26" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="E38" s="26" t="n">
         <v>30</v>
@@ -12552,7 +13079,7 @@
         <v>124</v>
       </c>
       <c r="D39" s="26" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="E39" s="26" t="n">
         <v>65</v>
@@ -12569,10 +13096,10 @@
         <v>132</v>
       </c>
       <c r="D40" s="26" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="E40" s="26" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12583,10 +13110,10 @@
         <v>85</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="D41" s="26" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="E41" s="26" t="n">
         <v>274</v>
@@ -12600,10 +13127,10 @@
         <v>85</v>
       </c>
       <c r="C42" s="26" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="D42" s="26" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="E42" s="26" t="n">
         <v>356</v>
@@ -12617,10 +13144,10 @@
         <v>85</v>
       </c>
       <c r="C43" s="26" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="D43" s="26" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="E43" s="26" t="n">
         <v>2</v>
@@ -12634,10 +13161,10 @@
         <v>85</v>
       </c>
       <c r="C44" s="26" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="D44" s="26" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="E44" s="26" t="n">
         <v>100</v>
@@ -12651,11 +13178,11 @@
         <v>79</v>
       </c>
       <c r="C45" s="26" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D45" s="26"/>
       <c r="E45" s="26" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -12682,77 +13209,77 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="50" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="51" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="51" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="51" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="51" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="51" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="51" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="51" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="51" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="51" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="51" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="51" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="49.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="51" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="51" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="51" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>